<commit_message>
onboarding: accept email/UPN for deploying identity; UAMI guardrails
Stage 1 now resolves a non-GUID deployingIdentity.objectId (email/UPN of a user, or appId/display name of a service principal) to the Entra objectId via az ad, so operators don't have to look up GUIDs. A GUID is kept verbatim; an unresolvable value fails with clear remediation.

Also: Stage 1 requires managedIdentity.id (FR1.1); Stage 4 adds UAMI pre-flight checks (existence Fail, role-assignment Warn); both planning forms gain a managedIdentity.id row and updated deployingIdentity.objectId notes; USER-GUIDE documents email/UPN support.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: 74389d48-0fb3-43bc-a3df-50ea8197a20b
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -807,7 +807,7 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Entra objectId of the identity that will deploy. FR1.0</t>
+          <t>Identity that will deploy (Stage 2 grants it the platform roles). Accepts either the Entra objectId (GUID), or - for convenience - an email/UPN of a user in the target tenant (or an app registration's appId/display name). Stage 1 resolves a non-GUID value to the objectId via 'az' (run 'az login' first). FR1.0</t>
         </is>
       </c>
     </row>
@@ -845,69 +845,69 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="6" customHeight="1" s="16"/>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+    <row r="14" ht="6" customHeight="1" s="16">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>managedIdentity.id</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>/subscriptions/&lt;subId&gt;/resourceGroups/&lt;rg&gt;/providers/Microsoft.ManagedIdentity/userAssignedIdentities/&lt;uami-name&gt;</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Pre-created User-Assigned Managed Identity (UAMI) resource id attached to the platform resources (supercomputer + workspace). This is NOT the deploying identity above; the tool does not create it. Required by Stage 4. FR4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>NETWORK</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>network.model</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>byo-existing</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>byo-existing = your VNet already exists; the tool does NOT build it (Stage 3 validates). Use 'byo' instead to have the tool provision subnets into your VNet. FR1.2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>network.networkResourceGroup</t>
+          <t>network.model</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>network-rg</t>
+          <t>byo-existing</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Resource group holding your existing (pre-created) VNet. FR1.2</t>
+          <t>byo-existing = your VNet already exists; the tool does NOT build it (Stage 3 validates). Use 'byo' instead to have the tool provision subnets into your VNet. FR1.2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>network.vnetCidr</t>
+          <t>network.networkResourceGroup</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>10.0.0.0/23</t>
+          <t>network-rg</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>VNet address space. FR1.2/FR1.3</t>
+          <t>Resource group holding your existing (pre-created) VNet. FR1.2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>network.spokeCidr</t>
+          <t>network.vnetCidr</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -917,102 +917,92 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
+          <t>VNet address space. FR1.2/FR1.3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>network.corpDns</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
+          <t>network.spokeCidr</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>10.0.0.0/23</t>
+        </is>
+      </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
+          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>network.nvaNextHop</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>10.1.0.4</t>
-        </is>
-      </c>
+          <t>network.corpDns</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n"/>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Firewall/NVA next-hop IP for forced tunneling; blank if none.</t>
+          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1" s="16">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>network.outboundType</t>
+          <t>network.nvaNextHop</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>UserDefinedRouting</t>
+          <t>10.1.0.4</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>AKS egress model: UserDefinedRouting (forced tunneling via nvaNextHop) | LoadBalancer (Azure-managed egress). FR1.2</t>
+          <t>Firewall/NVA next-hop IP for forced tunneling; blank if none.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
+          <t>network.outboundType</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>UserDefinedRouting</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>AKS egress model: UserDefinedRouting (forced tunneling via nvaNextHop) | LoadBalancer (Azure-managed egress). FR1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="6" customHeight="1" s="16">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
           <t>network.existingSubnets</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n"/>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="B24" s="12" t="n"/>
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>Comma-separated CIDRs already present in your existing VNet (besides the Discovery subnets below); Stage 1 checks the Discovery subnets do not overlap them. FR1.3</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="6" customHeight="1" s="16"/>
-    <row r="25" ht="43.75" customHeight="1" s="16">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="25" ht="43.75" customHeight="1" s="16"/>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>SUBNETS  (one SUBNET row per Discovery subnet: role, cidr, requiredPrefix, delegation)  FR1.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>aksSubnet</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.0/26</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>/26</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.ContainerService/managedClusters</t>
         </is>
       </c>
     </row>
@@ -1024,12 +1014,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>supercomputerNodepoolSubnet</t>
+          <t>aksSubnet</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>10.0.0.64/26</t>
+          <t>10.0.0.0/26</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -1039,7 +1029,7 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Microsoft.ContainerService/managedClusters</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1041,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>workspaceSubnet</t>
+          <t>supercomputerNodepoolSubnet</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>10.0.0.128/26</t>
+          <t>10.0.0.64/26</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1066,7 +1056,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Microsoft.App/environments</t>
+          <t>none</t>
         </is>
       </c>
     </row>
@@ -1078,12 +1068,12 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>agentSubnet</t>
+          <t>workspaceSubnet</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>10.0.0.192/26</t>
+          <t>10.0.0.128/26</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -1105,17 +1095,17 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>searchSubnet</t>
+          <t>agentSubnet</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>10.0.1.0/27</t>
+          <t>10.0.0.192/26</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>/27</t>
+          <t>/26</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -1132,12 +1122,12 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>privateEndpointSubnet</t>
+          <t>searchSubnet</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>10.0.1.32/27</t>
+          <t>10.0.1.0/27</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -1147,7 +1137,7 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Microsoft.App/environments</t>
         </is>
       </c>
     </row>
@@ -1159,301 +1149,311 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
+          <t>privateEndpointSubnet</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.32/27</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="6" customHeight="1" s="16">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
           <t>managementSubnet</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>10.0.1.64/27</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>/27</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="6" customHeight="1" s="16"/>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>STORAGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>storage.model</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>managed</t>
-        </is>
-      </c>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>byo | managed</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>storage.account</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="n"/>
+          <t>storage.model</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>managed</t>
+        </is>
+      </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>Existing storage account name (byo only).</t>
+          <t>byo | managed</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>storage.access</t>
+          <t>storage.account</t>
         </is>
       </c>
       <c r="B37" s="12" t="n"/>
       <c r="E37" s="13" t="inlineStr">
         <is>
+          <t>Existing storage account name (byo only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="6" customHeight="1" s="16">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>storage.access</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
           <t>Managed-storage network access: privateEndpoint | serviceEndpoint. Ignored when storage.model=byo.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="6" customHeight="1" s="16"/>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t>SIZING &amp; SCALE</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
-        <is>
-          <t>sizingTier</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>Small | Medium | Large (expands to quota/SKU). FR1.5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>bookshelf.inScope</t>
+          <t>sizingTier</t>
         </is>
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>true if Bookshelf indexing is deployed.</t>
+          <t>Small | Medium | Large (expands to quota/SKU). FR1.5</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>bookshelf.instances</t>
+          <t>bookshelf.inScope</t>
         </is>
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>Number of Bookshelf instances (&gt;=0).</t>
+          <t>true if Bookshelf indexing is deployed.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>bookshelf.instances</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>Project count; drives Cosmos RU/s = 2400 + 400 x projects. FR1.5</t>
+          <t>Number of Bookshelf instances (&gt;=0).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
+          <t>projects</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Project count; drives Cosmos RU/s = 2400 + 400 x projects. FR1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="6" customHeight="1" s="16">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
           <t>deployMode</t>
         </is>
       </c>
-      <c r="B44" s="12" t="n"/>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="B45" s="12" t="n"/>
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>Azure OpenAI model deployment type: GlobalStandard (default) | DataZoneStandard (keeps inference in-region for data residency). FR1.5.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="6" customHeight="1" s="16"/>
-    <row r="46" ht="29.15" customHeight="1" s="16">
-      <c r="A46" s="21" t="inlineStr">
+    <row r="46" ht="29.15" customHeight="1" s="16"/>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>NAMES  (per-type naming rules enforced in FR1.6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>names.workspace</t>
-        </is>
-      </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>disc-ws</t>
-        </is>
-      </c>
-      <c r="E47" s="13" t="inlineStr">
-        <is>
-          <t>3-24; also the endpoint subdomain; end with letter/digit.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>names.project</t>
+          <t>names.workspace</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>project1</t>
+          <t>disc-ws</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>3-12.</t>
+          <t>3-24; also the endpoint subdomain; end with letter/digit.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>names.supercomputer</t>
+          <t>names.project</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>disc-sc</t>
+          <t>project1</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>3-24.</t>
+          <t>3-12.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="17" t="inlineStr">
         <is>
-          <t>names.nodePool</t>
+          <t>names.supercomputer</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>pool1</t>
+          <t>disc-sc</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>3-12.</t>
+          <t>3-24.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
         <is>
-          <t>names.tool</t>
+          <t>names.nodePool</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>hero-tool</t>
+          <t>pool1</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>3-24.</t>
+          <t>3-12.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
         <is>
-          <t>names.agent</t>
+          <t>names.tool</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>hero-agent</t>
+          <t>hero-tool</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>3-63.</t>
+          <t>3-24.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="17" t="inlineStr">
         <is>
-          <t>names.storageContainer</t>
+          <t>names.agent</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>kb-container</t>
+          <t>hero-agent</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>3-24.</t>
+          <t>3-63.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="17" t="inlineStr">
         <is>
-          <t>names.storageAsset</t>
+          <t>names.storageContainer</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>kb-asset</t>
+          <t>kb-container</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -1465,58 +1465,75 @@
     <row r="55">
       <c r="A55" s="17" t="inlineStr">
         <is>
+          <t>names.storageAsset</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>kb-asset</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>3-24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="6" customHeight="1" s="16">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
           <t>names.investigation</t>
         </is>
       </c>
-      <c r="B55" s="12" t="n"/>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="B56" s="12" t="n"/>
+      <c r="E56" s="13" t="inlineStr">
         <is>
           <t>Name of the hero investigation created during Stage 5 scenario enablement (3-20 chars; default hero-inv). FR1.6/FR5.4.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="6" customHeight="1" s="16"/>
-    <row r="57" ht="29.15" customHeight="1" s="16">
-      <c r="A57" s="21" t="inlineStr">
+    <row r="57" ht="29.15" customHeight="1" s="16"/>
+    <row r="58" ht="25.75" customHeight="1" s="16">
+      <c r="A58" s="21" t="inlineStr">
         <is>
           <t>POLICY SET  (auto-collected from the subscription at runtime; FR1.7). Leave blank to use live assignments; add a POLICY row (Value = policy display name) only to declare/override one.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="25.75" customHeight="1" s="16">
-      <c r="A58" s="20" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B58" s="12" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+      <c r="B59" s="12" t="n"/>
+    </row>
+    <row r="60" ht="6" customHeight="1" s="16">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B59" s="12" t="n"/>
-      <c r="E59" s="13" t="n"/>
-    </row>
-    <row r="60" ht="6" customHeight="1" s="16"/>
-    <row r="61" ht="43.75" customHeight="1" s="16">
-      <c r="A61" s="21" t="inlineStr">
+      <c r="B60" s="12" t="n"/>
+      <c r="E60" s="13" t="n"/>
+    </row>
+    <row r="61" ht="43.75" customHeight="1" s="16"/>
+    <row r="62">
+      <c r="A62" s="21" t="inlineStr">
         <is>
           <t>WAIVERS  (one WAIVER row per overridden P0 check: checkId, justification, approvedBy)  FR1.8</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="20" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="20" t="inlineStr">
         <is>
           <t>WAIVER</t>
         </is>
       </c>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
+      <c r="B63" s="12" t="n"/>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
onboarding: E2E managed-VNet fixes (subnet delegation, UAMI roles, quota, reports)
- Stage 1: network.vnetName, guest-email identity fallback, role normalization,
  optional names, vCPU quota check; aksSubnet must not be delegated.
- Stage 2: artifact output dir follows -JsonPath.
- Stage 3: managedcluster subnet expects no delegation; management (spare) subnet
  delegated only for UserDefinedRouting; fallback checks Pass with reason.
- Stage 4: strict UAMI required-role gate, subnet-topology preflight, optional
  managementSubnetId (UDR only), nested ARM error details, quota and
  InternalServerError remediation rules, multiple -ReadinessReport inputs,
  missing $supercomputerId assignment, explained failure for empty resource id.
- Stage 5: remove in-VNet ephemeral VM connectivity probe (to move to Stage 3).
- Forms, schema, examples, specs and USER-GUIDE updated to match.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
@@ -365,6 +365,26 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>onboarding-tool</author>
+  </authors>
+  <commentList>
+    <comment ref="E29" authorId="0" shapeId="0">
+      <text>
+        <t>Must be none. The supercomputer system nodes run in this subnet; delegating it to Microsoft.ContainerService/managedClusters makes supercomputer creation fail with InternalServerError (target=internalMetadata).</t>
+      </text>
+    </comment>
+    <comment ref="E35" authorId="0" shapeId="0">
+      <text>
+        <t>AKS API-server VNet integration subnet. Used only when network.outboundType=UserDefinedRouting (must be delegated to Microsoft.ContainerService/managedClusters). With LoadBalancer it is reserved/unused.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -654,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -671,7 +691,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" s="16">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Fill the Value column (yellow). Column A tags are stable — do not rename. SUBNET/POLICY/WAIVER rows may be added or removed. Yellow example values are illustrative; overwrite them.</t>
@@ -702,14 +722,14 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" s="16">
       <c r="A5" s="21" t="inlineStr">
         <is>
           <t>IDENTITY &amp; SUBSCRIPTION</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" s="16">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>schemaVersion</t>
@@ -743,428 +763,408 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="25.75" customHeight="1" s="16">
       <c r="A8" s="17" t="inlineStr">
         <is>
+          <t>resourceGroup</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>platform-rg</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Resource group for the Discovery platform resources (supercomputer, workspace, project, chat model). Create it first (az group create); the pre-created UAMI usually lives here too. If blank, the tool uses network.networkResourceGroup. FR4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="16">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
           <t>environment</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>devtest</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>devtest | prod</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+    <row r="10" s="16">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>controlPlaneRegion</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>eastus2</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Azure short name for the control-plane region. FR1.1/FR1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>workloadRegion</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>eastus2</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Azure short name for the workload/data-plane region. FR1.4</t>
         </is>
       </c>
     </row>
     <row r="11" ht="25.75" customHeight="1" s="16">
       <c r="A11" s="17" t="inlineStr">
         <is>
+          <t>workloadRegion</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Azure short name for the workload/data-plane region. FR1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.75" customHeight="1" s="16">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
           <t>deployingIdentity.objectId</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000000</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Identity that will deploy (Stage 2 grants it the platform roles). Accepts either the Entra objectId (GUID), or - for convenience - an email/UPN of a user in the target tenant (or an app registration's appId/display name). Stage 1 resolves a non-GUID value to the objectId via 'az' (run 'az login' first). FR1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>deployingIdentity.type</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>user | servicePrincipal | managedIdentity</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25.75" customHeight="1" s="16">
       <c r="A13" s="17" t="inlineStr">
         <is>
+          <t>deployingIdentity.type</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>user | servicePrincipal | managedIdentity</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="25.75" customHeight="1" s="16">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
           <t>deployingIdentity.canRegisterProviders</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>true if it holds Contributor/Owner or .../register/action. FR1.0</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="6" customHeight="1" s="16">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="15" ht="25.75" customHeight="1" s="16">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>managedIdentity.id</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>/subscriptions/&lt;subId&gt;/resourceGroups/&lt;rg&gt;/providers/Microsoft.ManagedIdentity/userAssignedIdentities/&lt;uami-name&gt;</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>Pre-created User-Assigned Managed Identity (UAMI) resource id attached to the platform resources (supercomputer + workspace). This is NOT the deploying identity above; the tool does not create it. Required by Stage 4. FR4.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Pre-created User-Assigned Managed Identity (UAMI) resource id attached to the platform resources (supercomputer + workspace). This is NOT the deploying identity above; the tool does not create it (az identity create ... --query id -o tsv). Required (Stage 1 + Stage 4). FR4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="6" customHeight="1" s="16"/>
+    <row r="17" s="16">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>NETWORK</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="18" s="16">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>network.model</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>byo-existing</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>byo-existing = your VNet already exists; the tool does NOT build it (Stage 3 validates). Use 'byo' instead to have the tool provision subnets into your VNet. FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+    <row r="19" s="16">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>network.networkResourceGroup</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>network-rg</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Resource group holding your existing (pre-created) VNet. FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+    <row r="20" s="16">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>network.vnetName</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>my-existing-vnet</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Name of your EXISTING VNet in network.networkResourceGroup (the tool does not create it; Stage 1 checks it exists and is in controlPlaneRegion). Leave blank only if it is named vnet-&lt;names.workspace&gt;. FR1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="16">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>network.vnetCidr</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>10.0.0.0/23</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>VNet address space. FR1.2/FR1.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>network.spokeCidr</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.0/23</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>network.corpDns</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1" s="16">
       <c r="A22" s="17" t="inlineStr">
         <is>
+          <t>network.spokeCidr</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>10.0.0.0/23</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="16">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>network.corpDns</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="16">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
           <t>network.nvaNextHop</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>10.1.0.4</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>Firewall/NVA next-hop IP for forced tunneling; blank if none.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+    <row r="25" ht="24" customHeight="1" s="16">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>network.outboundType</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>UserDefinedRouting</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t>AKS egress model: UserDefinedRouting (forced tunneling via nvaNextHop) | LoadBalancer (Azure-managed egress). FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="6" customHeight="1" s="16">
-      <c r="A24" s="17" t="inlineStr">
+    <row r="26" ht="6" customHeight="1" s="16">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>network.existingSubnets</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="B26" s="12" t="n"/>
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>Comma-separated CIDRs already present in your existing VNet (besides the Discovery subnets below); Stage 1 checks the Discovery subnets do not overlap them. FR1.3</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="43.75" customHeight="1" s="16"/>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+    <row r="27" ht="6" customHeight="1" s="16"/>
+    <row r="28" ht="43.75" customHeight="1" s="16">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>SUBNETS  (one SUBNET row per Discovery subnet: role, cidr, requiredPrefix, delegation)  FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="29" s="16">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>aksSubnet</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>10.0.0.0/26</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>/26</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.ContainerService/managedClusters</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" s="16">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>supercomputerNodepoolSubnet</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>10.0.0.64/26</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>/26</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+    <row r="31" s="16">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>workspaceSubnet</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>10.0.0.128/26</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>/26</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Microsoft.App/environments</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+    <row r="32" s="16">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>agentSubnet</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>10.0.0.192/26</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>/26</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>Microsoft.App/environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>searchSubnet</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>10.0.1.0/27</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.App/environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>privateEndpointSubnet</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>10.0.1.32/27</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>none</t>
         </is>
       </c>
     </row>
@@ -1176,405 +1176,463 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
+          <t>searchSubnet</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.0/27</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.App/environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="6" customHeight="1" s="16">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>privateEndpointSubnet</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.32/27</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="6" customHeight="1" s="16">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
           <t>managementSubnet</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>10.0.1.64/27</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>/27</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.ContainerService/managedClusters</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="6" customHeight="1" s="16"/>
+    <row r="37" s="16">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>STORAGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>storage.model</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>managed</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>byo | managed</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>storage.account</t>
-        </is>
-      </c>
-      <c r="B37" s="12" t="n"/>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>Existing storage account name (byo only).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="6" customHeight="1" s="16">
       <c r="A38" s="17" t="inlineStr">
         <is>
+          <t>storage.model</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>managed</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>byo | managed</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="6" customHeight="1" s="16">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>storage.account</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Existing storage account name (byo only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="6" customHeight="1" s="16">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
           <t>storage.access</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="B40" s="12" t="n"/>
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>Managed-storage network access: privateEndpoint | serviceEndpoint. Ignored when storage.model=byo.</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+    <row r="41" ht="6" customHeight="1" s="16"/>
+    <row r="42" s="16">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>SIZING &amp; SCALE</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+    <row r="43" s="16">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>sizingTier</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E43" s="13" t="inlineStr">
         <is>
           <t>Small | Medium | Large (expands to quota/SKU). FR1.5</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+    <row r="44" s="16">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>bookshelf.inScope</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E44" s="13" t="inlineStr">
         <is>
           <t>true if Bookshelf indexing is deployed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>bookshelf.instances</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>Number of Bookshelf instances (&gt;=0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>projects</t>
-        </is>
-      </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>Project count; drives Cosmos RU/s = 2400 + 400 x projects. FR1.5</t>
         </is>
       </c>
     </row>
     <row r="45" ht="6" customHeight="1" s="16">
       <c r="A45" s="17" t="inlineStr">
         <is>
+          <t>bookshelf.instances</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Number of Bookshelf instances (&gt;=0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="6" customHeight="1" s="16">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>projects</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>Project count; drives Cosmos RU/s = 2400 + 400 x projects. FR1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="6" customHeight="1" s="16">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
           <t>deployMode</t>
         </is>
       </c>
-      <c r="B45" s="12" t="n"/>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="B47" s="12" t="n"/>
+      <c r="E47" s="13" t="inlineStr">
         <is>
           <t>Azure OpenAI model deployment type: GlobalStandard (default) | DataZoneStandard (keeps inference in-region for data residency). FR1.5.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="29.15" customHeight="1" s="16"/>
-    <row r="47">
-      <c r="A47" s="21" t="inlineStr">
+    <row r="48" ht="6" customHeight="1" s="16"/>
+    <row r="49" ht="29.15" customHeight="1" s="16">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>NAMES  (per-type naming rules enforced in FR1.6)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+    <row r="50" s="16">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>names.workspace</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>disc-ws</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>3-24; also the endpoint subdomain; end with letter/digit.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+    <row r="51" s="16">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>names.project</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>project1</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>3-12.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="17" t="inlineStr">
+    <row r="52" s="16">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>names.supercomputer</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>disc-sc</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+    <row r="53" s="16">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>names.nodePool</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>pool1</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E53" s="13" t="inlineStr">
         <is>
           <t>3-12.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+    <row r="54" s="16">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>names.tool</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>hero-tool</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
+      <c r="E54" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
+    <row r="55" s="16">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>names.agent</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>hero-agent</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E55" s="13" t="inlineStr">
         <is>
           <t>3-63.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
-        <is>
-          <t>names.storageContainer</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>kb-container</t>
-        </is>
-      </c>
-      <c r="E54" s="13" t="inlineStr">
-        <is>
-          <t>3-24.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>names.storageAsset</t>
-        </is>
-      </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>kb-asset</t>
-        </is>
-      </c>
-      <c r="E55" s="13" t="inlineStr">
-        <is>
-          <t>3-24.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="6" customHeight="1" s="16">
       <c r="A56" s="17" t="inlineStr">
         <is>
+          <t>names.storageContainer</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>kb-container</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>3-24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="6" customHeight="1" s="16">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>names.storageAsset</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>kb-asset</t>
+        </is>
+      </c>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>3-24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="6" customHeight="1" s="16">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
           <t>names.investigation</t>
         </is>
       </c>
-      <c r="B56" s="12" t="n"/>
-      <c r="E56" s="13" t="inlineStr">
+      <c r="B58" s="12" t="n"/>
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>Name of the hero investigation created during Stage 5 scenario enablement (3-20 chars; default hero-inv). FR1.6/FR5.4.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="29.15" customHeight="1" s="16"/>
-    <row r="58" ht="25.75" customHeight="1" s="16">
-      <c r="A58" s="21" t="inlineStr">
+    <row r="59" ht="6" customHeight="1" s="16"/>
+    <row r="60" ht="29.15" customHeight="1" s="16">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>POLICY SET  (auto-collected from the subscription at runtime; FR1.7). Leave blank to use live assignments; add a POLICY row (Value = policy display name) only to declare/override one.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="20" t="inlineStr">
+    <row r="61" ht="25.75" customHeight="1" s="16">
+      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B59" s="12" t="n"/>
-    </row>
-    <row r="60" ht="6" customHeight="1" s="16">
-      <c r="A60" s="17" t="inlineStr">
+      <c r="B61" s="12" t="n"/>
+    </row>
+    <row r="62" ht="6" customHeight="1" s="16">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B60" s="12" t="n"/>
-      <c r="E60" s="13" t="n"/>
-    </row>
-    <row r="61" ht="43.75" customHeight="1" s="16"/>
-    <row r="62">
-      <c r="A62" s="21" t="inlineStr">
+      <c r="B62" s="12" t="n"/>
+      <c r="E62" s="13" t="n"/>
+    </row>
+    <row r="63" ht="6" customHeight="1" s="16"/>
+    <row r="64" ht="43.75" customHeight="1" s="16">
+      <c r="A64" s="21" t="inlineStr">
         <is>
           <t>WAIVERS  (one WAIVER row per overridden P0 check: checkId, justification, approvedBy)  FR1.8</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="20" t="inlineStr">
+    <row r="65" s="16">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>WAIVER</t>
         </is>
       </c>
-      <c r="B63" s="12" t="n"/>
-      <c r="C63" s="12" t="n"/>
-      <c r="D63" s="12" t="n"/>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
-  <dataValidations count="8">
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="9">
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"devtest,prod"</formula1>
     </dataValidation>
-    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"user,servicePrincipal,managedIdentity"</formula1>
     </dataValidation>
-    <dataValidation sqref="B13 B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B14 B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B16 B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"managed,byo-existing,byo,byo-spoke,greenfield"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"byo,managed"</formula1>
     </dataValidation>
-    <dataValidation sqref="E26 E27 E28 E29 E30 E31 E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E29 E30 E31 E32 E33 E34 E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Microsoft.App/environments,Microsoft.ContainerService/managedClusters,none"</formula1>
     </dataValidation>
-    <dataValidation sqref="B37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"privateEndpoint,serviceEndpoint"</formula1>
     </dataValidation>
-    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Small,Medium,Large"</formula1>
     </dataValidation>
-    <dataValidation sqref="B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GlobalStandard,DataZoneStandard"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
onboarding: accept email/UPN for deploying identity + UAMI guardrails (#221)
Co-authored-by: leijgao <leijiagao@microsoft.com>
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: 74389d48-0fb3-43bc-a3df-50ea8197a20b
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
@@ -365,6 +365,26 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>onboarding-tool</author>
+  </authors>
+  <commentList>
+    <comment ref="E29" authorId="0" shapeId="0">
+      <text>
+        <t>Must be none. The supercomputer system nodes run in this subnet; delegating it to Microsoft.ContainerService/managedClusters makes supercomputer creation fail with InternalServerError (target=internalMetadata).</t>
+      </text>
+    </comment>
+    <comment ref="E35" authorId="0" shapeId="0">
+      <text>
+        <t>AKS API-server VNet integration subnet. Used only when network.outboundType=UserDefinedRouting (must be delegated to Microsoft.ContainerService/managedClusters). With LoadBalancer it is reserved/unused.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -654,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -671,7 +691,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" s="16">
       <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Fill the Value column (yellow). Column A tags are stable — do not rename. SUBNET/POLICY/WAIVER rows may be added or removed. Yellow example values are illustrative; overwrite them.</t>
@@ -702,14 +722,14 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" s="16">
       <c r="A5" s="21" t="inlineStr">
         <is>
           <t>IDENTITY &amp; SUBSCRIPTION</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" s="16">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>schemaVersion</t>
@@ -743,821 +763,876 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="25.75" customHeight="1" s="16">
       <c r="A8" s="17" t="inlineStr">
         <is>
+          <t>resourceGroup</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>platform-rg</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Resource group for the Discovery platform resources (supercomputer, workspace, project, chat model). Create it first (az group create); the pre-created UAMI usually lives here too. If blank, the tool uses network.networkResourceGroup. FR4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" s="16">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
           <t>environment</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>devtest</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>devtest | prod</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+    <row r="10" s="16">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>controlPlaneRegion</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>eastus2</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Azure short name for the control-plane region. FR1.1/FR1.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>workloadRegion</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>eastus2</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Azure short name for the workload/data-plane region. FR1.4</t>
         </is>
       </c>
     </row>
     <row r="11" ht="25.75" customHeight="1" s="16">
       <c r="A11" s="17" t="inlineStr">
         <is>
+          <t>workloadRegion</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Azure short name for the workload/data-plane region. FR1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.75" customHeight="1" s="16">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
           <t>deployingIdentity.objectId</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000000</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>Entra objectId of the identity that will deploy. FR1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>deployingIdentity.type</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>user | servicePrincipal | managedIdentity</t>
+          <t>Identity that will deploy (Stage 2 grants it the platform roles). Accepts either the Entra objectId (GUID), or - for convenience - an email/UPN of a user in the target tenant (or an app registration's appId/display name). Stage 1 resolves a non-GUID value to the objectId via 'az' (run 'az login' first). FR1.0</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25.75" customHeight="1" s="16">
       <c r="A13" s="17" t="inlineStr">
         <is>
+          <t>deployingIdentity.type</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>user | servicePrincipal | managedIdentity</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="25.75" customHeight="1" s="16">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
           <t>deployingIdentity.canRegisterProviders</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>true if it holds Contributor/Owner or .../register/action. FR1.0</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="6" customHeight="1" s="16"/>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+    <row r="15" ht="25.75" customHeight="1" s="16">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>managedIdentity.id</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>/subscriptions/&lt;subId&gt;/resourceGroups/&lt;rg&gt;/providers/Microsoft.ManagedIdentity/userAssignedIdentities/&lt;uami-name&gt;</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Pre-created User-Assigned Managed Identity (UAMI) resource id attached to the platform resources (supercomputer + workspace). This is NOT the deploying identity above; the tool does not create it (az identity create ... --query id -o tsv). Required (Stage 1 + Stage 4). FR4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="6" customHeight="1" s="16"/>
+    <row r="17" s="16">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>NETWORK</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+    <row r="18" s="16">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>network.model</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>byo-existing</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>byo-existing = your VNet already exists; the tool does NOT build it (Stage 3 validates). Use 'byo' instead to have the tool provision subnets into your VNet. FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="19" s="16">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>network.networkResourceGroup</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>network-rg</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Resource group holding your existing (pre-created) VNet. FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+    <row r="20" s="16">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>network.vnetName</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>my-existing-vnet</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Name of your EXISTING VNet in network.networkResourceGroup (the tool does not create it; Stage 1 checks it exists and is in controlPlaneRegion). Leave blank only if it is named vnet-&lt;names.workspace&gt;. FR1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="16">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>network.vnetCidr</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>10.0.0.0/23</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>VNet address space. FR1.2/FR1.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>network.spokeCidr</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.0/23</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>network.corpDns</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>network.nvaNextHop</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>10.1.0.4</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>Firewall/NVA next-hop IP for forced tunneling; blank if none.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1" s="16">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>network.outboundType</t>
+          <t>network.spokeCidr</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>UserDefinedRouting</t>
+          <t>10.0.0.0/23</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>AKS egress model: UserDefinedRouting (forced tunneling via nvaNextHop) | LoadBalancer (Azure-managed egress). FR1.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+          <t>Spoke/allocatable range if narrower than the VNet; else same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="16">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>network.existingSubnets</t>
+          <t>network.corpDns</t>
         </is>
       </c>
       <c r="B23" s="12" t="n"/>
       <c r="E23" s="13" t="inlineStr">
         <is>
+          <t>Comma-separated custom DNS server IPs; blank = Azure-provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="16">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>network.nvaNextHop</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>10.1.0.4</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Firewall/NVA next-hop IP for forced tunneling; blank if none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1" s="16">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>network.outboundType</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>UserDefinedRouting</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>AKS egress model: UserDefinedRouting (forced tunneling via nvaNextHop) | LoadBalancer (Azure-managed egress). FR1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="6" customHeight="1" s="16">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>network.existingSubnets</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n"/>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
           <t>Comma-separated CIDRs already present in your existing VNet (besides the Discovery subnets below); Stage 1 checks the Discovery subnets do not overlap them. FR1.3</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="6" customHeight="1" s="16"/>
-    <row r="25" ht="43.75" customHeight="1" s="16">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="27" ht="6" customHeight="1" s="16"/>
+    <row r="28" ht="43.75" customHeight="1" s="16">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>SUBNETS  (one SUBNET row per Discovery subnet: role, cidr, requiredPrefix, delegation)  FR1.2</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="29" s="16">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>SUBNET</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>aksSubnet</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>10.0.0.0/26</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>/26</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" s="16">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>supercomputerNodepoolSubnet</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>10.0.0.64/26</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>/26</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" s="16">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>workspaceSubnet</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>10.0.0.128/26</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>/26</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.App/environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" s="16">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>agentSubnet</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>10.0.0.192/26</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>/26</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.App/environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="6" customHeight="1" s="16">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>searchSubnet</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.0/27</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Microsoft.App/environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="6" customHeight="1" s="16">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>privateEndpointSubnet</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.32/27</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="6" customHeight="1" s="16">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>SUBNET</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>managementSubnet</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>10.0.1.64/27</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>/27</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Microsoft.ContainerService/managedClusters</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>supercomputerNodepoolSubnet</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.64/26</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>/26</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>workspaceSubnet</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.128/26</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>/26</t>
-        </is>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.App/environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>agentSubnet</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>10.0.0.192/26</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>/26</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.App/environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>searchSubnet</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>10.0.1.0/27</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>Microsoft.App/environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>privateEndpointSubnet</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>10.0.1.32/27</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>SUBNET</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>managementSubnet</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>10.0.1.64/27</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>/27</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="6" customHeight="1" s="16"/>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+    <row r="36" ht="6" customHeight="1" s="16"/>
+    <row r="37" s="16">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>STORAGE</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+    <row r="38" ht="6" customHeight="1" s="16">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>storage.model</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>managed</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E38" s="13" t="inlineStr">
         <is>
           <t>byo | managed</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+    <row r="39" ht="6" customHeight="1" s="16">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>storage.account</t>
         </is>
       </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="B39" s="12" t="n"/>
+      <c r="E39" s="13" t="inlineStr">
         <is>
           <t>Existing storage account name (byo only).</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+    <row r="40" ht="6" customHeight="1" s="16">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>storage.access</t>
         </is>
       </c>
-      <c r="B37" s="12" t="n"/>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="B40" s="12" t="n"/>
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>Managed-storage network access: privateEndpoint | serviceEndpoint. Ignored when storage.model=byo.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="6" customHeight="1" s="16"/>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+    <row r="41" ht="6" customHeight="1" s="16"/>
+    <row r="42" s="16">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>SIZING &amp; SCALE</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+    <row r="43" s="16">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>sizingTier</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E43" s="13" t="inlineStr">
         <is>
           <t>Small | Medium | Large (expands to quota/SKU). FR1.5</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+    <row r="44" s="16">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>bookshelf.inScope</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E44" s="13" t="inlineStr">
         <is>
           <t>true if Bookshelf indexing is deployed.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+    <row r="45" ht="6" customHeight="1" s="16">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>bookshelf.instances</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>Number of Bookshelf instances (&gt;=0).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+    <row r="46" ht="6" customHeight="1" s="16">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>projects</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>Project count; drives Cosmos RU/s = 2400 + 400 x projects. FR1.5</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+    <row r="47" ht="6" customHeight="1" s="16">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>deployMode</t>
         </is>
       </c>
-      <c r="B44" s="12" t="n"/>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="B47" s="12" t="n"/>
+      <c r="E47" s="13" t="inlineStr">
         <is>
           <t>Azure OpenAI model deployment type: GlobalStandard (default) | DataZoneStandard (keeps inference in-region for data residency). FR1.5.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="6" customHeight="1" s="16"/>
-    <row r="46" ht="29.15" customHeight="1" s="16">
-      <c r="A46" s="21" t="inlineStr">
+    <row r="48" ht="6" customHeight="1" s="16"/>
+    <row r="49" ht="29.15" customHeight="1" s="16">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>NAMES  (per-type naming rules enforced in FR1.6)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
+    <row r="50" s="16">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>names.workspace</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>disc-ws</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>3-24; also the endpoint subdomain; end with letter/digit.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+    <row r="51" s="16">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>names.project</t>
         </is>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>project1</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>3-12.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+    <row r="52" s="16">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>names.supercomputer</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>disc-sc</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="17" t="inlineStr">
+    <row r="53" s="16">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>names.nodePool</t>
         </is>
       </c>
-      <c r="B50" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>pool1</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E53" s="13" t="inlineStr">
         <is>
           <t>3-12.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+    <row r="54" s="16">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>names.tool</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>hero-tool</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E54" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+    <row r="55" s="16">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>names.agent</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>hero-agent</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
+      <c r="E55" s="13" t="inlineStr">
         <is>
           <t>3-63.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
+    <row r="56" ht="6" customHeight="1" s="16">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>names.storageContainer</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>kb-container</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E56" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
+    <row r="57" ht="6" customHeight="1" s="16">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>names.storageAsset</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>kb-asset</t>
         </is>
       </c>
-      <c r="E54" s="13" t="inlineStr">
+      <c r="E57" s="13" t="inlineStr">
         <is>
           <t>3-24.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
+    <row r="58" ht="6" customHeight="1" s="16">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t>names.investigation</t>
         </is>
       </c>
-      <c r="B55" s="12" t="n"/>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="B58" s="12" t="n"/>
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>Name of the hero investigation created during Stage 5 scenario enablement (3-20 chars; default hero-inv). FR1.6/FR5.4.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="6" customHeight="1" s="16"/>
-    <row r="57" ht="29.15" customHeight="1" s="16">
-      <c r="A57" s="21" t="inlineStr">
+    <row r="59" ht="6" customHeight="1" s="16"/>
+    <row r="60" ht="29.15" customHeight="1" s="16">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>POLICY SET  (auto-collected from the subscription at runtime; FR1.7). Leave blank to use live assignments; add a POLICY row (Value = policy display name) only to declare/override one.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="25.75" customHeight="1" s="16">
-      <c r="A58" s="20" t="inlineStr">
+    <row r="61" ht="25.75" customHeight="1" s="16">
+      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B58" s="12" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+      <c r="B61" s="12" t="n"/>
+    </row>
+    <row r="62" ht="6" customHeight="1" s="16">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>POLICY</t>
         </is>
       </c>
-      <c r="B59" s="12" t="n"/>
-      <c r="E59" s="13" t="n"/>
-    </row>
-    <row r="60" ht="6" customHeight="1" s="16"/>
-    <row r="61" ht="43.75" customHeight="1" s="16">
-      <c r="A61" s="21" t="inlineStr">
+      <c r="B62" s="12" t="n"/>
+      <c r="E62" s="13" t="n"/>
+    </row>
+    <row r="63" ht="6" customHeight="1" s="16"/>
+    <row r="64" ht="43.75" customHeight="1" s="16">
+      <c r="A64" s="21" t="inlineStr">
         <is>
           <t>WAIVERS  (one WAIVER row per overridden P0 check: checkId, justification, approvedBy)  FR1.8</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="20" t="inlineStr">
+    <row r="65" s="16">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>WAIVER</t>
         </is>
       </c>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A17:E17"/>
   </mergeCells>
-  <dataValidations count="8">
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="9">
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"devtest,prod"</formula1>
     </dataValidation>
-    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"user,servicePrincipal,managedIdentity"</formula1>
     </dataValidation>
-    <dataValidation sqref="B13 B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B14 B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B16 B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"managed,byo-existing,byo,byo-spoke,greenfield"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"byo,managed"</formula1>
     </dataValidation>
-    <dataValidation sqref="E26 E27 E28 E29 E30 E31 E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E29 E30 E31 E32 E33 E34 E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Microsoft.App/environments,Microsoft.ContainerService/managedClusters,none"</formula1>
     </dataValidation>
-    <dataValidation sqref="B37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"privateEndpoint,serviceEndpoint"</formula1>
     </dataValidation>
-    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Small,Medium,Large"</formula1>
     </dataValidation>
-    <dataValidation sqref="B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GlobalStandard,DataZoneStandard"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
onboarding: E2E fixes and configurable workspace public network access
Fixes found during a clean managed-VNet end-to-end run: Stage 4 gate no longer polls to timeout when the workspace has no Foundry account; Stage 1 fails early when Bookshelf is in scope without a BYO storage account; Stage 2 creates storage containers through ARM so the storage firewall does not block it. Adds workspace.publicNetworkAccess (default Enabled) to the forms and config, applied by Stage 4 and probed by Stage 5 before any data-plane call.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: 4cb86271-8828-4df2-b93b-38fc612175d3
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>managed</t>
+          <t>byo</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>byo | managed</t>
+          <t>byo | managed. Bookshelf (bookshelf.inScope=true) requires byo with storage.account set.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       <c r="B39" s="12" t="n"/>
       <c r="E39" s="13" t="inlineStr">
         <is>
-          <t>Existing storage account name (byo only).</t>
+          <t>Storage account name for Bookshelf (byo). Stage 2 creates it in the network resource group if it does not exist.</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       <c r="B40" s="12" t="n"/>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>Managed-storage network access: privateEndpoint | serviceEndpoint. Ignored when storage.model=byo.</t>
+          <t>BYO storage network access: privateEndpoint | serviceEndpoint (default privateEndpoint). Ignored when storage.model=managed.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,23 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="6" customHeight="1" s="16"/>
+    <row r="48" ht="6" customHeight="1" s="16">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>workspace.publicNetworkAccess</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>Workspace data-plane public network access: Enabled (default) | Disabled. Disabled means Stage 5 must run from inside the VNet. FR1.2</t>
+        </is>
+      </c>
+    </row>
     <row r="49" ht="29.15" customHeight="1" s="16">
       <c r="A49" s="21" t="inlineStr">
         <is>
@@ -1594,15 +1610,15 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A64:E64"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A17:E17"/>
   </mergeCells>
-  <dataValidations count="9">
+  <dataValidations count="10">
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"devtest,prod"</formula1>
     </dataValidation>
@@ -1629,6 +1645,9 @@
     </dataValidation>
     <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GlobalStandard,DataZoneStandard"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Enabled,Disabled"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
onboarding: E2E fixes and configurable workspace public network access (#222)
Co-authored-by: leijgao <leijiagao@microsoft.com>
Copilot-Session: 4cb86271-8828-4df2-b93b-38fc612175d3
</commit_message>
<xml_diff>
--- a/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
+++ b/utilities/onboarding-tool/scripts/stage1-planning/discovery-resource-planning-form-byo-vnet.xlsx
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>managed</t>
+          <t>byo</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>byo | managed</t>
+          <t>byo | managed. Bookshelf (bookshelf.inScope=true) requires byo with storage.account set.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       <c r="B39" s="12" t="n"/>
       <c r="E39" s="13" t="inlineStr">
         <is>
-          <t>Existing storage account name (byo only).</t>
+          <t>Storage account name for Bookshelf (byo). Stage 2 creates it in the network resource group if it does not exist.</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       <c r="B40" s="12" t="n"/>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>Managed-storage network access: privateEndpoint | serviceEndpoint. Ignored when storage.model=byo.</t>
+          <t>BYO storage network access: privateEndpoint | serviceEndpoint (default privateEndpoint). Ignored when storage.model=managed.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,23 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="6" customHeight="1" s="16"/>
+    <row r="48" ht="6" customHeight="1" s="16">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>workspace.publicNetworkAccess</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>Workspace data-plane public network access: Enabled (default) | Disabled. Disabled means Stage 5 must run from inside the VNet. FR1.2</t>
+        </is>
+      </c>
+    </row>
     <row r="49" ht="29.15" customHeight="1" s="16">
       <c r="A49" s="21" t="inlineStr">
         <is>
@@ -1594,15 +1610,15 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A64:E64"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A17:E17"/>
   </mergeCells>
-  <dataValidations count="9">
+  <dataValidations count="10">
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"devtest,prod"</formula1>
     </dataValidation>
@@ -1629,6 +1645,9 @@
     </dataValidation>
     <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GlobalStandard,DataZoneStandard"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Enabled,Disabled"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>